<commit_message>
Clear ERP master demo data
</commit_message>
<xml_diff>
--- a/mock-db/erp_mock_database.xlsx
+++ b/mock-db/erp_mock_database.xlsx
@@ -400,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P3"/>
+  <dimension ref="A1:P1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -452,116 +452,16 @@
         <v>hasDefaultAddress</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>LG000155</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Ananya Ghosh</v>
-      </c>
-      <c r="C2" t="str">
-        <v>98300 14210</v>
-      </c>
-      <c r="D2" t="str">
-        <v>B2C</v>
-      </c>
-      <c r="E2" t="str">
-        <v>["VIP","In-store","Grooming"]</v>
-      </c>
-      <c r="F2">
-        <v>18</v>
-      </c>
-      <c r="G2">
-        <v>48620</v>
-      </c>
-      <c r="H2">
-        <v>2</v>
-      </c>
-      <c r="I2">
-        <v>2</v>
-      </c>
-      <c r="J2">
-        <v>96</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Lake Gardens</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Walk-in</v>
-      </c>
-      <c r="N2" t="str">
-        <v>2026-06-03</v>
-      </c>
-      <c r="O2" t="str">
-        <v>2026-06-19</v>
-      </c>
-      <c r="P2" t="str">
-        <v>TRUE</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>RJ000064</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Arjun Kennels</v>
-      </c>
-      <c r="C3" t="str">
-        <v>98310 76218</v>
-      </c>
-      <c r="D3" t="str">
-        <v>B2B</v>
-      </c>
-      <c r="E3" t="str">
-        <v>["Breeder","Wholesale","Repeat"]</v>
-      </c>
-      <c r="F3">
-        <v>31</v>
-      </c>
-      <c r="G3">
-        <v>184500</v>
-      </c>
-      <c r="H3">
-        <v>6</v>
-      </c>
-      <c r="I3">
-        <v>7</v>
-      </c>
-      <c r="J3">
-        <v>88</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Active</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Rajarhat</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Referral</v>
-      </c>
-      <c r="N3" t="str">
-        <v>2026-05-14</v>
-      </c>
-      <c r="O3" t="str">
-        <v>2026-06-18</v>
-      </c>
-      <c r="P3" t="str">
-        <v>TRUE</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:Y1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -640,170 +540,16 @@
         <v>lastSale</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>WHI-OCF-70G</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Ocean Fish Adult Dry Food</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Whiskas</v>
-      </c>
-      <c r="D2" t="str">
-        <v/>
-      </c>
-      <c r="E2" t="str">
-        <v>8901003107012</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Standard</v>
-      </c>
-      <c r="G2" t="str">
-        <v>pc</v>
-      </c>
-      <c r="H2">
-        <v>70</v>
-      </c>
-      <c r="I2" t="str">
-        <v>g</v>
-      </c>
-      <c r="J2" t="str">
-        <v>Food</v>
-      </c>
-      <c r="K2" t="str">
-        <v>Dry Food</v>
-      </c>
-      <c r="L2" t="str">
-        <v>["Cat"]</v>
-      </c>
-      <c r="M2" t="str">
-        <v>["Daily Care"]</v>
-      </c>
-      <c r="N2">
-        <v>65</v>
-      </c>
-      <c r="O2">
-        <v>62</v>
-      </c>
-      <c r="P2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>["Duplicate"]</v>
-      </c>
-      <c r="R2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="S2" t="str">
-        <v>Standard</v>
-      </c>
-      <c r="T2" t="str">
-        <v/>
-      </c>
-      <c r="U2" t="str">
-        <v>23091000</v>
-      </c>
-      <c r="V2" t="str">
-        <v>18</v>
-      </c>
-      <c r="W2" t="str">
-        <v>2025-11-14</v>
-      </c>
-      <c r="X2" t="str">
-        <v>2026-06-18</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>2026-06-20</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>RC-MAX-4KG</v>
-      </c>
-      <c r="B3" t="str">
-        <v>Maxi Adult Dry Food</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Royal Canin</v>
-      </c>
-      <c r="D3" t="str">
-        <v/>
-      </c>
-      <c r="E3" t="str">
-        <v>3182550402220</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Standard</v>
-      </c>
-      <c r="G3" t="str">
-        <v>bag</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-      <c r="I3" t="str">
-        <v>kg</v>
-      </c>
-      <c r="J3" t="str">
-        <v>Food</v>
-      </c>
-      <c r="K3" t="str">
-        <v>Dry Food</v>
-      </c>
-      <c r="L3" t="str">
-        <v>["Dog"]</v>
-      </c>
-      <c r="M3" t="str">
-        <v>["Premium","Daily Care"]</v>
-      </c>
-      <c r="N3">
-        <v>3250</v>
-      </c>
-      <c r="O3">
-        <v>3090</v>
-      </c>
-      <c r="P3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>[]</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Active</v>
-      </c>
-      <c r="S3" t="str">
-        <v>Standard</v>
-      </c>
-      <c r="T3" t="str">
-        <v/>
-      </c>
-      <c r="U3" t="str">
-        <v>23091000</v>
-      </c>
-      <c r="V3" t="str">
-        <v>18</v>
-      </c>
-      <c r="W3" t="str">
-        <v>2025-08-09</v>
-      </c>
-      <c r="X3" t="str">
-        <v>2026-05-30</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>2026-06-19</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Y3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Y1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:U3"/>
+  <dimension ref="A1:U1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -870,146 +616,16 @@
         <v>lastPerformed</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>SRV-GRM-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Full Grooming</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Grooming</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Haircut &amp; Styling</v>
-      </c>
-      <c r="E2" t="str">
-        <v>Grooming</v>
-      </c>
-      <c r="F2" t="str">
-        <v>["Groomer","Senior Groomer"]</v>
-      </c>
-      <c r="G2" t="str">
-        <v>["Dog","Cat"]</v>
-      </c>
-      <c r="H2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="I2">
-        <v>90</v>
-      </c>
-      <c r="J2">
-        <v>1800</v>
-      </c>
-      <c r="K2">
-        <v>1650</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Tiered</v>
-      </c>
-      <c r="M2">
-        <v>4</v>
-      </c>
-      <c r="N2" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="O2" t="str">
-        <v>[]</v>
-      </c>
-      <c r="P2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>["Popular","Premium"]</v>
-      </c>
-      <c r="R2" t="str">
-        <v>999729</v>
-      </c>
-      <c r="S2" t="str">
-        <v>18</v>
-      </c>
-      <c r="T2" t="str">
-        <v>2025-08-12</v>
-      </c>
-      <c r="U2" t="str">
-        <v>2026-06-21</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>SRV-VET-001</v>
-      </c>
-      <c r="B3" t="str">
-        <v>General Veterinary Consultation</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Veterinary Care</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Consultation</v>
-      </c>
-      <c r="E3" t="str">
-        <v>Veterinary</v>
-      </c>
-      <c r="F3" t="str">
-        <v>["Veterinarian","Veterinary Surgeon"]</v>
-      </c>
-      <c r="G3" t="str">
-        <v>["Dog","Cat"]</v>
-      </c>
-      <c r="H3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="I3">
-        <v>30</v>
-      </c>
-      <c r="J3">
-        <v>700</v>
-      </c>
-      <c r="K3">
-        <v>700</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Fixed</v>
-      </c>
-      <c r="M3">
-        <v>1</v>
-      </c>
-      <c r="N3" t="str">
-        <v>TRUE</v>
-      </c>
-      <c r="O3" t="str">
-        <v>[]</v>
-      </c>
-      <c r="P3" t="str">
-        <v>Active</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>["Popular"]</v>
-      </c>
-      <c r="R3" t="str">
-        <v>999316</v>
-      </c>
-      <c r="S3" t="str">
-        <v>18</v>
-      </c>
-      <c r="T3" t="str">
-        <v>2025-07-02</v>
-      </c>
-      <c r="U3" t="str">
-        <v>2026-06-22</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:U3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:U1"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:Q3"/>
+  <dimension ref="A1:Q1"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -1064,115 +680,9 @@
         <v>flags</v>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>VEN-001</v>
-      </c>
-      <c r="B2" t="str">
-        <v>Pawsome Distribution Pvt Ltd</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Pawsome Distribution Private Limited</v>
-      </c>
-      <c r="D2" t="str">
-        <v>Rohit Sharma</v>
-      </c>
-      <c r="E2" t="str">
-        <v>98300 44210</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Distributor</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Product</v>
-      </c>
-      <c r="H2" t="str">
-        <v>["Food","Healthcare"]</v>
-      </c>
-      <c r="I2" t="str">
-        <v>Registered</v>
-      </c>
-      <c r="J2" t="str">
-        <v>19AAJCP1234F1Z7</v>
-      </c>
-      <c r="K2" t="str">
-        <v>30 Days</v>
-      </c>
-      <c r="L2" t="str">
-        <v>Billing Date</v>
-      </c>
-      <c r="M2" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Kolkata</v>
-      </c>
-      <c r="O2" t="str">
-        <v>["Preferred","Credit"]</v>
-      </c>
-      <c r="P2" t="str">
-        <v>2026-06-04</v>
-      </c>
-      <c r="Q2" t="str">
-        <v>[]</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="str">
-        <v>VEN-003</v>
-      </c>
-      <c r="B3" t="str">
-        <v>VetCare Pharma Supplies</v>
-      </c>
-      <c r="C3" t="str">
-        <v>VetCare Pharma Supplies LLP</v>
-      </c>
-      <c r="D3" t="str">
-        <v>Dr. Arindam Basu</v>
-      </c>
-      <c r="E3" t="str">
-        <v>81001 66220</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Supplier</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Consumable</v>
-      </c>
-      <c r="H3" t="str">
-        <v>["Healthcare","Medicines"]</v>
-      </c>
-      <c r="I3" t="str">
-        <v>Registered</v>
-      </c>
-      <c r="J3" t="str">
-        <v>19AAVFV9900K1Z5</v>
-      </c>
-      <c r="K3" t="str">
-        <v>7 Days</v>
-      </c>
-      <c r="L3" t="str">
-        <v>Billing Date</v>
-      </c>
-      <c r="M3" t="str">
-        <v>Active</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Salt Lake</v>
-      </c>
-      <c r="O3" t="str">
-        <v>["Drug License"]</v>
-      </c>
-      <c r="P3" t="str">
-        <v>2025-12-12</v>
-      </c>
-      <c r="Q3" t="str">
-        <v>[]</v>
-      </c>
-    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:Q3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:Q1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>